<commit_message>
suppression contraintes + correctifs d0da3de3eaba28a295c2c48cf3944840e0a920d3
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgc-signature.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgc-signature.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-16T21:31:30+00:00</t>
+    <t>2026-07-17T08:00:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -4910,7 +4910,7 @@
         <v>79</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>73</v>
@@ -4985,7 +4985,7 @@
         <v>79</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>73</v>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G37" t="s" s="2">
         <v>79</v>
@@ -5388,7 +5388,7 @@
         <v>154</v>
       </c>
       <c r="AG37" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH37" t="s" s="2">
         <v>79</v>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G49" t="s" s="2">
         <v>79</v>
@@ -6600,7 +6600,7 @@
         <v>170</v>
       </c>
       <c r="AG49" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH49" t="s" s="2">
         <v>79</v>

</xml_diff>